<commit_message>
chore: Add versioning to all documents and scripts
This commit adds 'Version 2.0' to all relevant project files to improve maintainability and track changes.

The version number has been added to:
- The `Dashboard` sheet via the `create_excel_structure.py` script.
- The header comment of the `twilio_macro.vbs` script.
- The top of the `user_guide.md`.
- The top of the `developer_guide.md`.
</commit_message>
<xml_diff>
--- a/TwilioSender.xlsx
+++ b/TwilioSender.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,10 @@
       <b val="1"/>
       <color rgb="004F81BD"/>
       <sz val="18"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
     </font>
     <font>
       <b val="1"/>
@@ -77,14 +81,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -468,16 +475,21 @@
           <t>Twilio WhatsApp Messenger</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Version 2.0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>How to Use</t>
         </is>
       </c>
     </row>
     <row r="4" ht="100" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>1. Go to 'Settings' to enter your Twilio credentials.
 2. Go to 'Templates' to define your messages. Map a Message UID to a Twilio ContentSid and set the base variables.
@@ -488,30 +500,30 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Active Message UID:</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>PROMO_01</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Messages Per Second (MPS):</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
   </mergeCells>
@@ -529,97 +541,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>WhatsApp Number</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Send?</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{1}}</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{2}}</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{3}}</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{4}}</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{5}}</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{6}}</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{7}}</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{8}}</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{9}}</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{10}}</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{11}}</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{12}}</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{13}}</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{14}}</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Contact Variable {{15}}</t>
         </is>
@@ -770,87 +782,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Message UID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>ContentSid</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{1}}</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{2}}</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{3}}</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{4}}</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{5}}</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{6}}</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{7}}</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{8}}</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{9}}</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{10}}</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{11}}</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{12}}</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{13}}</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{14}}</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{15}}</t>
         </is>
@@ -934,32 +946,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Contact Number</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Message UID</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Twilio Response</t>
         </is>
@@ -980,12 +992,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>

</xml_diff>

<commit_message>
feat: Add reference columns to Templates sheet
This commit enhances the usability of the `Templates` sheet by adding several new columns for reference purposes.

The following columns have been added:
- `Description`: To provide a human-readable description of the template.
- `Template Content (Reference Only)`: To store the raw text of the Twilio template for easy viewing within Excel.
- `Sample Final Content (Preview)`: A programmatically generated column that shows a preview of the message with the 'Base Variables' filled in.

The Python script (`create_excel_structure.py`) has been updated to generate these new columns and the sample preview. The documentation has also been updated to explain their purpose. The VBA macro is unaffected as these columns are for reference only.
</commit_message>
<xml_diff>
--- a/TwilioSender.xlsx
+++ b/TwilioSender.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,75 +794,90 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Template Content (Reference Only)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Sample Final Content (Preview)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Base Variable {{1}}</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{2}}</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{3}}</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{4}}</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{5}}</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{6}}</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{7}}</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{8}}</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{9}}</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{10}}</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{11}}</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{12}}</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{13}}</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{14}}</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Base Variable {{15}}</t>
         </is>
@@ -881,55 +896,78 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Promotional offer for unutilized production capacity.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Special Offer: {{1}}
+Regular Price: ₹{{2}} | Your Discount: {{3}}%
+Offer valid from {{4}} to {{5}}.
+Visit us or connect today.
+{{6}}
+{{7}}
+(Attached: {{8}})</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Special Offer: {{contact_var_1}}
+Regular Price: ₹{{contact_var_2}} | Your Discount: {{contact_var_3}}%
+Offer valid from {{contact_var_4}} to {{contact_var_5}}.
+Visit us or connect today.
+{{contact_var_6}}
+{{contact_var_7}}
+(Attached: {{contact_var_8}})</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>{{contact_var_1}}</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>{{contact_var_2}}</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>{{contact_var_3}}</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>{{contact_var_4}}</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>{{contact_var_5}}</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>{{contact_var_6}}</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>{{contact_var_7}}</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>{{contact_var_8}}</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>{{contact_var_9}}</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>